<commit_message>
chore(masterdata): Dodge 4b 튜닝 — 슬리퍼 4 m/s, 스테이지 세기(1 0.8 / 3 1.6·0.8 / 4 2.3·0.8 / 5 1.4)
목표 A(보통 사람은 스테이지 3~4에서, 판 1~2분). 봇 측정: 탈락 2 10% · 3 40% · 4 13% · 5 30% · SD 7%, 중앙값 84초.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#DodgeStage.xlsx
+++ b/table/Datas/#DodgeStage.xlsx
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G5" t="n">
         <v>0.5</v>
@@ -651,10 +651,10 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="G7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H7" t="n">
         <v>1.5</v>
@@ -683,10 +683,10 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1.2</v>
+        <v>2.3</v>
       </c>
       <c r="G8" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H8" t="n">
         <v>1.6</v>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="G9" t="n">
         <v>0.6</v>

</xml_diff>